<commit_message>
Final fixes and improvements
</commit_message>
<xml_diff>
--- a/indicator.xlsx
+++ b/indicator.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,6 +486,11 @@
           <t>Обновлено_неделя</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Удалено</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -514,22 +519,25 @@
         <v>2454.85</v>
       </c>
       <c r="H2" t="n">
-        <v>293.42</v>
+        <v>292.67</v>
       </c>
       <c r="I2" t="n">
-        <v>2471.93</v>
+        <v>2470.47</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.02389557191609204</v>
+        <v>-0.02597747091134761</v>
       </c>
       <c r="K2" t="n">
-        <v>0.01115476667533088</v>
+        <v>0.009147148225615576</v>
       </c>
       <c r="L2" s="1" t="n">
         <v>46315</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>46315</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -559,22 +567,25 @@
         <v>2454.85</v>
       </c>
       <c r="H3" t="n">
-        <v>495.3</v>
+        <v>481.7</v>
       </c>
       <c r="I3" t="n">
-        <v>2471.93</v>
+        <v>2470.47</v>
       </c>
       <c r="J3" t="n">
-        <v>0.111558268732626</v>
+        <v>0.0792005561245277</v>
       </c>
       <c r="K3" t="n">
-        <v>0.05843275128515568</v>
+        <v>0.02977388938266845</v>
       </c>
       <c r="L3" s="1" t="n">
         <v>46315</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>46315</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -604,22 +615,25 @@
         <v>2454.85</v>
       </c>
       <c r="H4" t="n">
-        <v>0.722</v>
+        <v>0.681</v>
       </c>
       <c r="I4" t="n">
-        <v>2471.93</v>
+        <v>2470.47</v>
       </c>
       <c r="J4" t="n">
-        <v>0.07043722843319511</v>
+        <v>0.005164815728111227</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05014336963630517</v>
+        <v>-0.009291171917688468</v>
       </c>
       <c r="L4" s="1" t="n">
         <v>46315</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>46315</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>